<commit_message>
Complete curva cross-check: PROCV code column, summary by class, order descriptions
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H3XY78Wxyj9y6JPXoWJTyP
</commit_message>
<xml_diff>
--- a/PEDIDO_ESTHER_DIST_CLASSE.xlsx
+++ b/PEDIDO_ESTHER_DIST_CLASSE.xlsx
@@ -7587,7 +7587,10 @@
       <c r="C14" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="15"/>
+      <c r="D14" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C14," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE FREIO PEUGEOT</v>
+      </c>
       <c r="E14" s="18" t="n">
         <v>88</v>
       </c>
@@ -7618,7 +7621,10 @@
       <c r="C15" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="15"/>
+      <c r="D15" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C15," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE FREIO GM</v>
+      </c>
       <c r="E15" s="18" t="n">
         <v>113.19</v>
       </c>
@@ -7648,7 +7654,10 @@
       <c r="C16" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="15"/>
+      <c r="D16" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C16," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE FREIO FIAT/JEEP</v>
+      </c>
       <c r="E16" s="18" t="n">
         <v>220</v>
       </c>
@@ -7678,7 +7687,10 @@
       <c r="C17" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="D17" s="15"/>
+      <c r="D17" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C17," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE FREIO M BENZ</v>
+      </c>
       <c r="E17" s="18" t="n">
         <v>242</v>
       </c>
@@ -7708,7 +7720,10 @@
       <c r="C18" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="15"/>
+      <c r="D18" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C18," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE FREIO M BENZ</v>
+      </c>
       <c r="E18" s="18" t="n">
         <v>195.63</v>
       </c>
@@ -7738,7 +7753,10 @@
       <c r="C19" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="15"/>
+      <c r="D19" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C19," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE FREIO FIAT</v>
+      </c>
       <c r="E19" s="18" t="n">
         <v>143.99</v>
       </c>
@@ -7768,7 +7786,10 @@
       <c r="C20" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="D20" s="15"/>
+      <c r="D20" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C20," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE FREIO TOYOTA</v>
+      </c>
       <c r="E20" s="18" t="n">
         <v>266.75</v>
       </c>
@@ -7798,7 +7819,10 @@
       <c r="C21" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="15"/>
+      <c r="D21" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C21," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>BANDEJA COMPLETA LE FORD</v>
+      </c>
       <c r="E21" s="18" t="n">
         <v>150</v>
       </c>
@@ -7828,7 +7852,10 @@
       <c r="C22" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="D22" s="15"/>
+      <c r="D22" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C22," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>BANDEJA COMPLETA LD FORD</v>
+      </c>
       <c r="E22" s="18" t="n">
         <v>150</v>
       </c>
@@ -7858,7 +7885,10 @@
       <c r="C23" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="D23" s="15"/>
+      <c r="D23" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C23," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>BANDEJA COMPLETA LE FIAT</v>
+      </c>
       <c r="E23" s="18" t="n">
         <v>198</v>
       </c>
@@ -7888,7 +7918,10 @@
       <c r="C24" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="D24" s="15"/>
+      <c r="D24" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C24," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>BANDEJA COMPLETA LD FIAT</v>
+      </c>
       <c r="E24" s="18" t="n">
         <v>198</v>
       </c>
@@ -7918,7 +7951,10 @@
       <c r="C25" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="D25" s="15"/>
+      <c r="D25" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C25," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE EMBREAGEM TOYOTA</v>
+      </c>
       <c r="E25" s="18" t="n">
         <v>62</v>
       </c>
@@ -7948,7 +7984,10 @@
       <c r="C26" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="D26" s="15"/>
+      <c r="D26" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C26," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE EMBREAGEM HONDA</v>
+      </c>
       <c r="E26" s="18" t="n">
         <v>95</v>
       </c>
@@ -7978,7 +8017,10 @@
       <c r="C27" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D27" s="15"/>
+      <c r="D27" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C27," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE EMBREAGEM RENAULT</v>
+      </c>
       <c r="E27" s="18" t="n">
         <v>113.4</v>
       </c>
@@ -8008,7 +8050,10 @@
       <c r="C28" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="D28" s="15"/>
+      <c r="D28" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C28," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE EMBREAGEM MITSUBISHI</v>
+      </c>
       <c r="E28" s="22" t="n">
         <v>82.53</v>
       </c>
@@ -8038,7 +8083,10 @@
       <c r="C29" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="D29" s="15"/>
+      <c r="D29" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C29," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE EMBREAGEM TOYOTA</v>
+      </c>
       <c r="E29" s="23" t="n">
         <v>78.19</v>
       </c>
@@ -8068,7 +8116,10 @@
       <c r="C30" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="D30" s="15"/>
+      <c r="D30" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C30," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE EMBREAGEM NISSAN</v>
+      </c>
       <c r="E30" s="23" t="n">
         <v>95.8</v>
       </c>
@@ -8098,7 +8149,10 @@
       <c r="C31" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="D31" s="15"/>
+      <c r="D31" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C31," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>POLIA VISCOSA CASE</v>
+      </c>
       <c r="E31" s="18" t="n">
         <v>377.72</v>
       </c>
@@ -8128,7 +8182,10 @@
       <c r="C32" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="D32" s="15"/>
+      <c r="D32" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C32," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>RESFRIADOR OLEO JEEP</v>
+      </c>
       <c r="E32" s="18" t="n">
         <v>355.44</v>
       </c>
@@ -8158,7 +8215,10 @@
       <c r="C33" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="D33" s="15"/>
+      <c r="D33" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C33," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>RESFRIADRO DE ÓLEO MOTOR RENAULT</v>
+      </c>
       <c r="E33" s="18" t="n">
         <v>358.64</v>
       </c>
@@ -8188,7 +8248,10 @@
       <c r="C34" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="D34" s="15"/>
+      <c r="D34" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C34," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>RESFRIADOR DE ÓLEO RENAULT</v>
+      </c>
       <c r="E34" s="18" t="n">
         <v>574.99</v>
       </c>
@@ -8218,7 +8281,10 @@
       <c r="C35" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="D35" s="15"/>
+      <c r="D35" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C35," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO AUXILIAR DE EMBREAGEM TOYOTA</v>
+      </c>
       <c r="E35" s="23" t="n">
         <v>59.99</v>
       </c>
@@ -8248,7 +8314,10 @@
       <c r="C36" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="D36" s="15"/>
+      <c r="D36" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C36," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO DE RODA LE/LD FIAT</v>
+      </c>
       <c r="E36" s="23" t="n">
         <v>31.88</v>
       </c>
@@ -8278,7 +8347,10 @@
       <c r="C37" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="D37" s="15"/>
+      <c r="D37" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C37," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO DE RODA LE/LD FORD</v>
+      </c>
       <c r="E37" s="23" t="n">
         <v>26.99</v>
       </c>
@@ -8308,7 +8380,10 @@
       <c r="C38" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="D38" s="15"/>
+      <c r="D38" s="15" t="str">
+        <f aca="false">IFERROR(VLOOKUP(SUBSTITUTE($C38," ",""),Curva!$A:$E,2,0),"")</f>
+        <v>CILINDRO MESTRE DE EMBREAGEM VW</v>
+      </c>
       <c r="E38" s="23" t="n">
         <v>86.49</v>
       </c>

</xml_diff>